<commit_message>
youngle: below-the-fold content (explained benefits, expectation timeline, actives) on product pages, docs table; Mira inline product chip stays on one line
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/youngle-produktangaben.xlsx
+++ b/docs/youngle-produktangaben.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Youngle Produktangaben" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Weiterführende Inhalte" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +29,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -55,12 +59,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1896,4 +1901,1062 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Handle (unser Shop)</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Produktvorteile erklärt</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Was kannst du erwarten (Einleitung)</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Was kannst du erwarten (Phasen)</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Wirkstoffe (Einleitung)</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Wirkstoffe (Name · Dosis · Aussage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>akg-calcium-alphaketoglutarat</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützt einen stabilen und gut regulierten Stoffwechsel
+Alpha-Ketoglutarat ist ein natürlicher Bestandteil des Energiestoffwechsels und an wichtigen Stoffwechselkreisläufen beteiligt. Es unterstützt Prozesse, die Nährstoffverwertung, Energiegewinnung und metabolische Steuerung miteinander verbinden. So entsteht eine stabile Basis, auf der der Stoffwechsel ruhig und effizient arbeiten kann.
+Fördert gleichmäßige Energie auf Zellebene
+Zelluläre Energie entsteht in den Mitochondrien und muss kontinuierlich bereitgestellt werden. AKG ist direkt in diese Prozesse eingebunden und unterstützt eine gleichmäßige Energieverwertung im Zellstoffwechsel. Energie steht dadurch verlässlich zur Verfügung, ohne das System zu stimulieren oder zu überfordern.
+Stärkt die strukturelle Stabilität und Qualität von Zellen
+Zellen müssen ihre Struktur und Funktion über lange Zeiträume erhalten. AKG unterstützt Prozesse, die an Anpassung, Stabilität und zellulärer Qualität beteiligt sind. Dadurch bleiben zentrale Zellfunktionen auch unter Belastung und mit zunehmendem Alter besser erhalten.
+Unterstützt nachhaltige Vitalität und gesundes Altern
+Langfristige Vitalität entsteht nicht durch kurzfristige Effekte, sondern durch gut abgestimmte Energiesysteme und stabile Zellfunktionen. Die gezielte Unterstützung dieser Prozesse durch AKG wirkt systemisch und über die Zeit. So entsteht eine verlässliche Grundlage für gesundes Altern und nachhaltige Leistungsfähigkeit.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie AKG zentrale Stoffwechselwege und die zelluläre Regeneration kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen wird AKG in zentrale Stoffwechselprozesse eingebunden, die an Energieverwertung und metabolischer Regulation beteiligt sind. Auf zellulärer Ebene beginnt die Unterstützung von Kreisläufen, die Nährstoffverarbeitung und Energiefluss miteinander verbinden. Spürbare Effekte stehen in dieser frühen Phase nicht im Vordergrund, da AKG nicht stimulierend wirkt.
+4 Wochen
+Mit fortgesetzter Einnahme können sich die unterstützten Stoffwechselprozesse stabilisieren. Der Körper reagiert häufig gleichmäßiger auf Ernährung, Aktivität und Belastung. Im Alltag äußert sich dies weniger als einzelner Effekt, sondern als ein ruhigeres, konstanteres Energie- und Belastungsniveau.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Anwendung greifen energetische und regulatorische Prozesse verlässlicher ineinander. Die Zusammenarbeit von Stoffwechsel, Mitochondrien und zellulären Erhaltungsmechanismen wirkt besser abgestimmt. Viele Anwender berichten in dieser Phase von einer insgesamt stabileren Leistungsfähigkeit ohne ausgeprägte Schwankungen.
+6 Monate
+AKG entfaltet seine Wirkung vor allem langfristig über die Unterstützung grundlegender Stoffwechsel- und Zellprozesse. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als eine stabile metabolische Basis. Die kontinuierliche Begleitung dieser Systeme trägt dazu bei, Vitalität und Belastbarkeit über die Zeit zu erhalten.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Diese Foundation basiert auf einem Wirkstoff, der auf zentrale zelluläre Mechanismen wirkt, die mit gesundem Altern in Verbindung stehen.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Calcium-Alpha-Ketoglutarat (AKG) · 1.000 mg · Unterstützt kontinuierliche mitochondriale ATP-Bereitstellung. Stabilisiert zelluläre Energieflüsse ohne Stimulation. Beteiligt an epigenetischer Enzymregulation. Beeinflusst altersassoziierte Zellfunktionen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>apigenin-kapseln</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Fördert stabile mitochondriale Leistung ohne Stimulation
+Energieversorgung auf Zellebene muss gleichmäßig und reguliert ablaufen. Apigenin unterstützt die funktionelle Stabilität mitochondrialer Prozesse, ohne stimulierend in den Energiestoffwechsel einzugreifen. So bleibt Energie verfügbar, ohne das System zu überreizen.
+Begleitet energieabhängige Anpassungs- und Regenerationsprozesse
+Regeneration und Anpassung benötigen kontrollierten Energieeinsatz, nicht maximale Aktivierung. Apigenin begleitet Prozesse, die Energie gezielt für Reparatur und Erholung einsetzen. Dadurch können Anpassungsmechanismen geordnet ablaufen.
+Stärkt den Erhalt von NAD⁺ im Zellstoffwechsel
+NAD⁺ ist essenziell für Energiegewinnung und zelluläre Reparatur. Apigenin wirkt regulierend auf Prozesse, die den NAD⁺-Verbrauch beeinflussen. So bleibt der NAD⁺-Haushalt auch unter Belastung besser im Gleichgewicht.
+Unterstützt nachhaltige Vitalität und gesundes Altern
+Langfristige Vitalität beruht auf stabilen, nicht überreizten Energiesystemen. Die regulierende Begleitung zentraler Energie- und Reparaturprozesse trägt dazu bei, Leistungsfähigkeit über die Zeit zu bewahren. So entsteht eine ruhige Grundlage für gesundes Altern.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Apigenin entzündungsmodulierende Signalwege und die zelluläre Stressresilienz kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen wird Apigenin in zelluläre Prozesse eingebunden, die den Umgang mit Stress und Energieverbrauch regulieren. Besonders abends unterstützt es ausgleichende Mechanismen im Energiestoffwechsel. Viele Menschen nehmen in dieser Phase ein ruhigeres Abschalten oder ein stabileres nächtliches Erholungsgefühl wahr, ohne sedierende Effekte.
+4 Wochen
+Mit fortgesetzter Einnahme können sich die regulierenden Effekte auf mitochondriale Leistung und energieabhängige Anpassungsprozesse deutlicher zeigen. Energie wird gleichmäßiger genutzt, insbesondere in Phasen von Regeneration und Erholung. Im Alltag äußert sich dies häufig in stabilerer Belastbarkeit und weniger innerer Unruhe.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Anwendung greifen die unterstützten Regulationsmechanismen verlässlicher ineinander. Der Umgang mit energetischer Belastung wirkt geordneter, Regenerationsprozesse können effizienter ablaufen. Viele Anwender berichten in dieser Phase von einem insgesamt ruhigeren Leistungsniveau und verbesserter Erholungsqualität.
+6 Monate
+Apigenin entfaltet seine Wirkung vor allem langfristig über die Begleitung zentraler Energie- und Schutzprozesse auf Zellebene. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als eine nachhaltige Stabilisierung der zellulären Energiegrundlage. Die regulierende Unterstützung des NAD⁺-Haushalts und mitochondrialer Funktionen trägt dazu bei, Vitalität und Anpassungsfähigkeit über die Zeit zu bewahren.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Diese Foundation basiert auf einem Wirkstoff, der auf zentrale zelluläre Mechanismen wirkt, die mit gesundem Altern in Verbindung stehen.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Apigenin · 100 mg · Stabilisiert mitochondriale Energieprozesse. Wirkt regulierend auf zellulären Energiestoffwechsel. Hemmt NAD⁺-verbrauchende Enzymaktivität. Stabilisiert NAD⁺-abhängige Reparatursysteme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>berberin-kapseln</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Hilft, starke Schwankungen im Energie- und Zuckerstoffwechsel auszugleichen
+Moderne Ernährungsgewohnheiten und unregelmäßige Mahlzeiten stellen hohe Anforderungen an den Zuckerstoffwechsel. Berberin unterstützt physiologische Prozesse, die an der Regulation von Glukose- und Energieverwertung beteiligt sind. So können ausgeprägte Schwankungen im Tagesverlauf besser ausgeglichen werden.
+Fördert metabolische Balance bei moderner Ernährung und Stress
+Ernährung, Stress und Schlaf beeinflussen den Stoffwechsel täglich. Berberin unterstützt regulatorische Mechanismen, die helfen, diese Belastungen einzuordnen. Dadurch bleibt die metabolische Balance auch unter wechselnden Anforderungen erhalten.
+Unterstützt einen stabilen Stoffwechsel und gleichmäßige Energie im Alltag
+Ein stabil arbeitender Stoffwechsel ist die Grundlage für konstante Energie. Durch die Unterstützung zentraler Stoffwechselprozesse kann Energie gleichmäßiger bereitgestellt werden. So entstehen weniger Leistungstiefs im Alltag.
+Unterstützt langfristige Stoffwechselgesundheit und gesundes Altern
+Langfristige Stoffwechselgesundheit beruht auf verlässlichen Regulationsprozessen. Die gezielte Unterstützung dieser Systeme trägt dazu bei, Energie, Balance und Belastbarkeit über die Zeit zu bewahren. So entsteht eine nachhaltige Grundlage für gesundes Altern.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Berberin den Glukose- und Lipidstoffwechsel sowie metabolische Regulationsprozesse kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen beginnt Berberin, in regulatorische Prozesse des Glukose- und Energiestoffwechsels einzugreifen. Auf physiologischer Ebene werden Mechanismen unterstützt, die den Umgang mit Zucker und Energie nach Mahlzeiten beeinflussen. Manche Menschen nehmen bereits in dieser Phase weniger ausgeprägte Energieeinbrüche oder ein stabileres Gefühl nach dem Essen wahr.
+4 Wochen
+Mit fortgesetzter Einnahme können sich die regulierenden Effekte auf den Stoffwechsel deutlicher etablieren. Schwankungen im Energie- und Zuckerstoffwechsel treten häufig weniger stark auf. Im Alltag zeigt sich dies oft in konstanterer Energie über den Tag hinweg, insbesondere bei wechselnden Mahlzeiten oder stressbedingten Belastungen.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Anwendung greifen metabolische Regulationsmechanismen verlässlicher ineinander. Viele Anwender berichten in dieser Phase von einer insgesamt besseren metabolischen Balance, weniger Leistungstiefs und einer stabileren Reaktion auf Ernährung und Stress. Der Stoffwechsel wirkt belastbarer und gleichmäßiger gesteuert.
+6 Monate
+Berberin entfaltet seine Wirkung vor allem über die langfristige Unterstützung zentraler Stoffwechselprozesse. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als ein insgesamt stabilerer metabolischer Zustand. Die kontinuierliche Begleitung von Glukose- und Fettstoffwechsel trägt dazu bei, Stoffwechselgesundheit und Energieverfügbarkeit über die Zeit zu erhalten.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Diese Foundation basiert auf einem Wirkstoff, der auf zentrale zelluläre Mechanismen wirkt, die mit gesundem Altern in Verbindung stehen.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Berberin-Hydrochlorid · 500 mg · Moduliert zelluläre Glukoseverwertung. Stabilisiert metabolische Signalachsen. Reguliert insulinabhängige Signalübertragung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>essentials-formula</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Stabilisiert zentrale Energie- und Erhaltungsprozesse der Zelle
+Energie- und Erhaltungsprozesse der Zelle müssen kontinuierlich und im Gleichgewicht ablaufen. Magnesium wirkt als Cofaktor der ATP-Produktion und der enzymatischen Reaktionen, die die tägliche Zellfunktion aufrechterhalten. Vitamin B12 und B6 unterstützen den Energiestoffwechsel und den laufenden enzymatischen Unterhalt der Zelle. Gemeinsam schaffen sie ein stabiles Fundament für essenzielle Zellfunktionen.
+Fördert die Zellerneuerung durch regulierte Recyclingprozesse
+Zellerneuerung beruht auf dem konstanten, regulierten Wiederaufbau dessen, was die Zelle abbaut. 5-MTHF-Folat speist aktives Folat direkt in die Methylierungs- und DNA-Synthesewege hinter der Zellteilung ein. Methylcobalamin arbeitet als bioaktive B12-Form an seiner Seite und hält denselben Ein-Kohlenstoff-Zyklus in Bewegung. Gemeinsam sichern sie eine ununterbrochene Erneuerung und Zellteilung.
+Setzt durchgängig auf hochwertige, gut verwertbare Nährstoffformen
+Ein Nährstoff wirkt nur so gut, wie der Körper ihn aufnehmen kann. Essentials⁺ setzt deshalb durchgängig auf die bioaktiven und chelatierten Formen: Magnesium und Zink als Bisglycinat-Chelate für hohe Aufnahme bei guter Magenverträglichkeit, Folat als 5-MTHF und B12 als Methylcobalamin in ihrer direkt verwertbaren Form, K2 als all-trans-MK-7. Gemeinsam sorgen sie dafür, dass ankommt, was auf dem Etikett steht.
+Unterstützt langfristige Vitalität und gesundes Altern
+Langfristige Vitalität hängt davon ab, wie gut der Körper seine Ressourcen über die Jahre lenkt. Vitamin D3 erhöht die Calcium-Verfügbarkeit und unterstützt Immun- und Bewegungsapparat. K2 MK-7 all-trans aktiviert die Proteine, die dieses Calcium in den Knochen und aus den Arterien heraus steuern. Gemeinsam legen sie das Fundament für eine Vitalität, die über die Zeit trägt.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Essentials⁺ die tägliche Grundversorgung sicherstellt und zentrale Körperfunktionen kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen treten die enthaltenen Mikronährstoffe in ihre jeweiligen zellulären Prozesse ein. Magnesium, B6 und B12 beginnen, den Energiestoffwechsel und den enzymatischen Unterhalt zu unterstützen, während Zink, Selen und Kupfer in die antioxidativen und Reparatursysteme einfließen. Folat und B12 füllen den Methylierungszyklus auf, und D3 mit K2 MK-7 beginnen, die Calcium-Regulation zu unterstützen. Spürbare Effekte stehen in dieser frühen Phase nicht im Vordergrund. Vielmehr wird die zelluläre Versorgung schrittweise ins Gleichgewicht gebracht.
+4 Wochen
+Bei fortgesetzter Einnahme erreichen die enzymatischen und metabolischen Systeme, die auf diese Mikronährstoffe angewiesen sind, eine gleichmäßigere Sättigung. Magnesium, B6 und B12 stützen den Energiestoffwechsel konstanter, der Methylierungszyklus läuft mit einer volleren Folat- und B12-Versorgung, und die antioxidativen Enzyme haben verlässlichen Zugriff auf ihre Cofaktoren Zink, Selen und Kupfer. Im Alltag zeigt sich das oft weniger als einzelner Effekt, sondern als stabilere Grundlage von Energie, Belastbarkeit und Regeneration.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Einnahme verschieben sich messbare Statusmarker. Die Serumspiegel von B12, Folat und Selen pendeln sich in einem volleren Bereich ein, und die Vitamin-D-Speicher bauen sich schrittweise zu einer stabilen Versorgung auf. Mit dem Schließen der zugrunde liegenden Defizite arbeiten die Systeme, die diese Nährstoffe speisen, aus einem gesicherten statt einem randständigen Fundament. Das gilt für Energiestoffwechsel, Zellerneuerung und antioxidativen Schutz gleichermaßen. Viele beschreiben diese Phase als verlässlichere innere Balance, mit gleichmäßigerer Energie und effizienterer Regeneration.
+6 Monate
+Essentials⁺ entfaltet seine volle Stärke als gefüllte, gepflegte Nährstoffbasis. Nach mehreren Monaten geht es nicht mehr um einen einzelnen Nährstoff, sondern um ein Fundament, auf das sich jede nachgelagerte Zellfunktion verlassen kann, mit aufgefüllten Vitamin-D-Speichern, verlässlich versorgter Methylierung und vollständig ausgestatteten antioxidativen Systemen. Genau das macht Essentials⁺ zur Basisschicht des gesamten Youngle-Systems. Es sichert die Grundlagen, damit gezielte Formeln auf festem Boden aufbauen können, ohne tägliche Feinjustierung.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Essentials⁺ wurde entwickelt, um die häufigsten ernährungsbedingten Defizite gezielt auszugleichen und die tägliche Grundversorgung mit essenziellen Vitaminen und Mineralstoffen sicherzustellen.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Vitamin D3 (Cholecalciferol) · 50 µg · Reguliert vitamin-D-abhängige Genexpression. Moduliert hormonelle Signalwege.
+Selen · 55 µg · Ermöglicht selenabhängige antioxidative Enzymaktivität. Beeinflusst immunologische Redoxbalance.
+Vitamin B12 · 500 µg · Unterstützt neurologische Funktion
+Magnesium-Bisglycinat · 150 mg · Unterstützt die normale Nervenfunktion. Trägt zur Stabilität nächtlicher Ruhephasen bei
+Zink · 15 mg · Reguliert zelluläre Signalwege der Immunantwort. Unterstützt Funktion immunologischer Enzymsysteme.
+Vitamin K2 (MK-7) · 200 µg · Moduliert inflammationsassoziierte Signalprozesse. Beeinflusst altersabhängige Gefäß- und Zellprozesse.
+Folat · 400 µg · Unterstützt Ein-Kohlenstoff-Stoffwechsel. Beteiligt an methylierungsabhängiger Hormonregulation.
+Vitamin B6 (Pyridoxin) · 2 mg · Beteiligt an hormonabhängiger Neurotransmitter-Synthese.
+Kupfer · 1 mg · Bestandteil antioxidativer Metalloenzyme. Beteiligt an zellulären Immunfunktionen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>fem-formula</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützt hormonelle Balance und natürliche Regulationsprozesse
+DIM unterstützt hormonelle Stoffwechselwege, die für Balance und Regulation entscheidend sind. Vitamin B6, Folat und Vitamin B12 tragen zu normalen hormonellen Funktionen bei und unterstützen die natürliche hormonelle Regulation des Körpers.
+Hilft, Stressbelastung besser zu bewältigen und innere Stabilität zu fördern
+Ashwagandha unterstützt die Anpassungsfähigkeit des Körpers bei körperlicher und mentaler Belastung. Magnesium ergänzt diese Wirkung, indem es zur normalen Funktion von Nerven und Muskeln beiträgt. Dadurch kann innere Stabilität auch in anspruchsvollen Phasen erhalten bleiben.
+Fördert zyklusbezogenes Wohlbefinden und emotionale Ausgeglichenheit
+Das Erleben des Zyklus entsteht aus einem fein abgestimmten hormonellen Zusammenspiel. DIM begleitet diese Prozesse und unterstützt ein harmonischeres Erleben des Zyklus. Vitamin B6, Folat und Vitamin B12 fördern emotionale Stabilität und helfen, zyklusbedingte Schwankungen besser auszugleichen.
+Unterstützt Knochengesundheit und hormonelle Stabilität im gesunden Altern
+Calcium und Vitamin D3 spielen eine zentrale Rolle für die Erhaltung normaler Knochen. In Verbindung mit einer ausgewogenen hormonellen Regulation entsteht strukturelle Stabilität über die Zeit. So wird eine nachhaltige Grundlage für gesundes Altern unterstützt.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Fem⁺ hormonelle Regulationsprozesse, Nährstoffbalance und geschlechtsspezifische Stoffwechselfunktionen kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen beginnen Ashwagandha, Magnesium und B-Vitamine, auf stress- und nervensystembezogene Regulationsprozesse einzuwirken. Viele Frauen nehmen in dieser Phase ein ruhigeres inneres Grundgefühl oder weniger Spannung wahr. Spürbare hormonelle Veränderungen stehen noch nicht im Vordergrund, erste Effekte betreffen vor allem emotionale Stabilität.
+4 Wochen
+Mit fortgesetzter Einnahme über einen vollständigen Zyklus können sich hormonelle Regulationsprozesse gleichmäßiger einpendeln. DIM begleitet den Östrogenstoffwechsel, während Vitamin D3, Calcium und Magnesium zyklusabhängige Anforderungen unterstützen. Im Alltag berichten viele Frauen von stabilerer Stimmung, weniger ausgeprägten Schwankungen und verbessertem zyklusbezogenem Wohlbefinden.
+3 Monate
+Nach mehreren Zyklen kontinuierlicher Anwendung können sich die unterstützten Regulationsmechanismen deutlicher auswirken. Zyklusverlauf, Energieempfinden und emotionale Belastbarkeit fühlen sich häufig verlässlicher an. In dieser Phase entsteht oft ein besseres Körpergefühl für hormonelle Rhythmen und individuelle Bedürfnisse.
+6 Monate
+FEM⁺ ist auf langfristige Begleitung ausgelegt, muss jedoch nicht dauerhaft ohne Unterbrechung eingenommen werden. Viele Frauen entscheiden sich nach mehreren Monaten bewusst für eine zyklusabhängige oder phasenweise Anwendung, etwa in Zeiten erhöhter Belastung oder hormoneller Veränderung. Die zuvor unterstützten Regulationsprozesse können dabei als stabile Grundlage erhalten bleiben.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Fem⁺ wurde entwickelt, um zentrale hormonelle Prozesse zu unterstützen und die physiologische Balance im weiblichen Körper zu fördern.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>DIM (Diindolylmethan) · 100 mg · Moduliert Östrogen-Stoffwechselwege. Beeinflusst hormonelle Regulationsprozesse.
+Ashwagandha-Extrakt · 300 mg · Moduliert Stressantwort des Körpers. Beeinflusst hypothalamisch-hypophysäre Achse.
+Calcium · 300 mg · Ermöglicht calciumabhängige Zell-Signaltransduktion. Beteiligt an hormoneller Freisetzungsregulation.
+Magnesium · 45 mg · Beteiligt an neuromuskulärer Signalübertragung. Moduliert neuronale Erregbarkeit.
+Vitamin D3 (Cholecalciferol) · 50 µg · Reguliert vitamin-D-abhängige Genexpression. Moduliert hormonelle Signalwege.
+Folat · 200 µg · Unterstützt Ein-Kohlenstoff-Stoffwechsel. Beteiligt an methylierungsabhängiger Hormonregulation.
+Vitamin B12 (Cobalamin) · 100 µg · Ermöglicht methylierungsabhängige Stoffwechselprozesse. Beteiligt an neuroendokriner Regulation.
+Vitamin B6 (Pyridoxin) · 2 mg · Beteiligt an hormonabhängiger Neurotransmitter-Synthese.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>focus-formula</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützt konzentriertes Arbeiten und mentale Klarheit im Alltag
+CDP-Cholin und Phosphatidylserin unterstützen zentrale Prozesse der neuronalen Signalübertragung. Sie tragen dazu bei, geistige Klarheit und Fokus im Alltag aufrechtzuerhalten. So wird konzentriertes Arbeiten auch bei komplexen Anforderungen erleichtert.
+Fördert geistige Ausdauer und stabile Leistungsfähigkeit über den Tag hinweg
+Lion’s Mane unterstützt neuronale Strukturen, die für nachhaltige kognitive Leistungsfähigkeit relevant sind. L-Taurin ergänzt diese Wirkung, indem es ausgleichende Prozesse im Nervensystem fördert. Dadurch kann mentale Leistungsfähigkeit gleichmäßiger über den Tag bestehen bleiben.
+Hilft, mentale Ermüdung bei anhaltender kognitiver Belastung zu reduzieren
+Anhaltende geistige Beanspruchung stellt hohe Anforderungen an das Nervensystem. B-Vitamine wie B6, Folat und B12 unterstützen den Energiestoffwechsel der Nervenzellen. So kann mentale Ermüdung bei längerer Belastung besser ausgeglichen werden.
+Unterstützt langfristige Gehirngesundheit und kognitive Stabilität
+Kognitive Leistungsfähigkeit beruht auf stabilen neuronalen Strukturen und einer verlässlichen Versorgung des Nervensystems. Die gezielte Kombination ausgewählter Inhaltsstoffe unterstützt Prozesse, die geistige Balance und kognitive Stabilität fördern. So entsteht eine nachhaltige Grundlage für mentale Leistungsfähigkeit über die Zeit.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Focus⁺ kognitive Leistungsfähigkeit, mentale Klarheit und neuronale Signalprozesse kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+Bereits in den ersten Tagen beginnen Taurin, CDP-Cholin und B-Vitamine, Prozesse der neuronalen Energieversorgung und Signalübertragung zu unterstützen. Viele Menschen nehmen eine verbesserte geistige Klarheit, ruhigere Konzentration oder weniger mentale Zerstreuung wahr. Die Wirkung setzt ohne stimulierende Effekte wie Nervosität oder innere Unruhe ein.
+4 Wochen
+Mit fortgesetzter Einnahme über mehrere Wochen kann sich die mentale Leistungsfähigkeit weiter stabilisieren. Konzentrationsphasen fühlen sich häufig gleichmäßiger an, geistige Ermüdung bei längerer Belastung tritt weniger abrupt auf. Im Alltag zeigt sich dies oft in besserer Fokusfähigkeit bei Arbeit, Lernen oder komplexen Aufgaben.
+3 Monate
+Bei zeitlich begrenzter Anwendung über mehrere Monate können sich kognitive Routinen festigen. Lion’s Mane und Phosphatidylserin begleiten Prozesse, die mit neuronaler Anpassung und Stressverarbeitung verbunden sind. Viele Anwender berichten, dass sie Fokus und mentale Struktur in dieser Phase auch ohne tägliche Einnahme besser abrufen können.
+6 Monate
+Nach längerer Anwendung entscheiden sich viele Menschen bewusst für Pausen oder eine situative Nutzung, etwa in Phasen hoher geistiger Anforderungen. Die zuvor unterstützten kognitiven Prozesse können dabei als Grundlage für stabile mentale Leistungsfähigkeit erhalten bleiben.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Focus⁺ wurde entwickelt, um zentrale Prozesse der Hirnfunktion zu unterstützen und die neuronale Energieversorgung effizient zu fördern.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>L-Taurin · 600 mg · Reguliert neuronale Calcium-Homöostase Moduliert inhibitorische Neurotransmission
+Lion’s Mane Extrakt · 400 mg · Stimuliert Nervenwachstumsfaktor-Synthese. Unterstützt neuronale strukturelle Plastizität.
+CDP-Cholin · 300 mg · Unterstützt cholinerge Neurotransmission Unterstützt Aufmerksamkeit und mentale Verarbeitung
+Phosphatidylserin · 100 mg · Unterstützt neuronale Membranstruktur Assoziiert mit kognitiver Leistungsfähigkeit im Alter
+Vitamin B6 · 2 mg · Unterstützt neuronalen Energiestoffwechsel
+Folat · 200 µg · Unterstützt Zellstoffwechsel im Nervensystem
+Vitamin B12 · 500 µg · Unterstützt neurologische Funktion</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>glycin-nac-kapseln</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützt die körpereigene Glutathionbildung und zelluläre Schutzmechanismen
+Der Körper kann Glutathion nur bilden, wenn ihm die richtigen Bausteine zur Verfügung stehen. Glycin und N-Acetyl-Cystein liefern genau diese Vorstufen, die im Alltag und mit zunehmendem Alter oft limitiert sind. So wird die körpereigene Fähigkeit unterstützt, zentrale Schutzmechanismen auf Zellebene aufrechtzuerhalten.
+Hilft, oxidativen Stress auszugleichen und die zelluläre Balance zu erhalten
+Im Alltag entstehen ständig oxidative Belastungen, etwa durch Stoffwechselprozesse, körperliche Aktivität, Stress oder Umwelteinflüsse. Glutathion hilft dabei, diese Belastungen auszugleichen und Zellen im inneren Gleichgewicht zu halten. GlyNAC unterstützt diesen Prozess, indem es die natürliche Redox-Balance des Körpers stabilisiert und so zur zellulären Balance beiträgt.
+Fördert die Regenerationsfähigkeit von Zellen bei metabolischer Belastung
+Wenn Zellen stärker gefordert sind, steigt auch der Bedarf an Reparatur- und Entlastungsprozessen. Glutathion spielt dabei eine wichtige Rolle, um Abbauprodukte zu verarbeiten und die Regeneration zu unterstützen. Durch die gezielte Versorgung mit Glycin und NAC bleibt diese Erholungsfähigkeit auch unter Belastung erhalten.
+Unterstützt langfristige Zellgesundheit und gesundes Altern
+Mit zunehmendem Alter nimmt die Fähigkeit des Körpers ab, zentrale Schutz- und Erneuerungsprozesse zuverlässig aufrechtzuerhalten. Eine stabile Glutathionversorgung gilt als wichtige Voraussetzung für langfristige Zellgesundheit. GlyNAC setzt genau hier an und unterstützt Prozesse, die helfen, zelluläre Funktion über die Zeit zu bewahren.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Glycin und NAC die körpereigene Glutathionbildung und den Schutz vor oxidativem Stress kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen stehen Glycin und N-Acetylcystein dem Körper als Vorstufen für die körpereigene Glutathionbildung zur Verfügung. Auf zellulärer Ebene werden antioxidative Schutzmechanismen unterstützt, ohne dass dies unmittelbar spürbar sein muss. Manche Menschen nehmen in dieser Phase ein ruhigeres körperliches Grundgefühl oder eine etwas bessere Erholung wahr.
+4 Wochen
+Mit fortgesetzter Einnahme kann sich die Unterstützung der Glutathionabhängigen Schutzsysteme stabilisieren. Zellen sind besser in der Lage, mit alltäglichen oxidativen Belastungen umzugehen. Im Alltag zeigt sich dies häufig weniger als einzelner Effekt, sondern als insgesamt ausgeglichenere Belastbarkeit und ein stabileres Energie- und Erholungsgefühl.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Versorgung greifen antioxidative Schutz- und Regenerationsprozesse verlässlicher ineinander. Die Fähigkeit von Zellen, mit metabolischem Stress umzugehen und Reparaturprozesse aufrechtzuerhalten, kann sich deutlich stabilisieren. Viele Anwender berichten in dieser Phase von besserer Regeneration, insbesondere bei körperlicher oder mentaler Belastung.
+6 Monate
+Glycin und N-Acetylcystein entfalten ihre Wirkung vor allem langfristig über die Unterstützung zentraler zellulärer Schutzmechanismen. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als eine insgesamt verbesserte zelluläre Widerstandskraft. Die kontinuierliche Begleitung der Glutathionbildung trägt dazu bei, Zellfunktion und Regenerationsfähigkeit über die Zeit zu erhalten.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Diese Foundation basiert auf Wirkstoffen, die auf zentrale zelluläre Mechanismen wirken, die mit gesundem Altern in Verbindung stehen.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>L-Glycin · 300 mg · Beteiligt an zellulären Reparaturprozessen. Liefert Glycin für Glutathion-Aufbau.
+N-Acetyl-Cystein (NAC) · 300 mg · Liefert Cystein für Glutathion-Biosynthese. Unterstützt thiolabhängige Zellschutzsysteme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>hyaluron-kapseln</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Fördert Gleitfähigkeit und Komfort von Gelenken und Bindegewebe
+Hyaluron ist ein zentraler Bestandteil der Gelenkflüssigkeit und wirkt dort als natürlicher Schmier- und Pufferstoff. Es unterstützt die viskoelastischen Eigenschaften, die für reibungsarme Bewegung entscheidend sind. So können Gelenke und umgebende Strukturen gleichmäßiger und komfortabler arbeiten.
+Trägt zur Hydration und Elastizität von Haut und Gewebe bei
+Hyaluron kann große Mengen Wasser binden und ist damit wesentlich für die Durchfeuchtung von Haut und Bindegewebe. Diese Eigenschaft trägt zur Elastizität und Spannkraft der Gewebestrukturen bei. So bleibt das Gewebe geschmeidig und widerstandsfähig.
+Stärkt die strukturelle Organisation zentraler Körpergewebe
+Als Bestandteil der extrazellulären Matrix beeinflusst Hyaluron den räumlichen Aufbau von Knorpel, Bindegewebe und Haut. Es unterstützt die Fähigkeit dieser Gewebe, Druck und Belastung gleichmäßig zu verteilen. Dadurch wird ihre funktionelle Stabilität gefördert.
+Unterstützt langfristige Gewebegesundheit und gesundes Altern
+Mit zunehmendem Alter nimmt der natürliche Hyalurongehalt vieler Gewebe ab. Die Unterstützung hyaluronabhängiger Strukturen trägt dazu bei, Beweglichkeit, Elastizität und Belastbarkeit über die Zeit zu erhalten. So entsteht eine verlässliche Grundlage für gesunde Gewebealterung.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Hyaluron die Hydration von Haut und Bindegewebe sowie die strukturelle Gewebeintegrität kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen wird Hyaluron in den Geweben verfügbar, die auf kontinuierliche Hydration und viskoelastische Eigenschaften angewiesen sind. Auf struktureller Ebene werden Prozesse unterstützt, die Wasserbindung und Gewebegleitfähigkeit betreffen. Spürbare Veränderungen sind in dieser frühen Phase nicht zwingend zu erwarten, manche Menschen nehmen jedoch ein angenehmeres Gefühl in Gelenken oder Haut wahr.
+4 Wochen
+Mit fortgesetzter Einnahme kann sich die hydratisierende Wirkung auf Gewebe deutlicher etablieren. Gelenkbewegungen fühlen sich häufig gleichmäßiger an, Haut und Bindegewebe können an Geschmeidigkeit gewinnen. Im Alltag zeigt sich dies weniger als einzelner Effekt, sondern als insgesamt verbessertes Komfort- und Bewegungsgefühl.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Versorgung greifen strukturelle Prozesse verlässlicher ineinander. Die Fähigkeit von Geweben, Wasser zu binden und Belastungen gleichmäßig zu verteilen, kann sich stabilisieren. Viele Anwender berichten in dieser Phase von besserer Beweglichkeit, elastischerem Hautgefühl und einem insgesamt stabileren Gewebeempfinden.
+6 Monate
+Hyaluron entfaltet seine Wirkung vor allem langfristig über die Unterstützung der strukturellen Organisation von Geweben. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als die Erhaltung von Elastizität, Gleitfähigkeit und Belastbarkeit. Die kontinuierliche Begleitung hyaluronabhängiger Strukturen trägt dazu bei, Gewebegesundheit und Funktion über die Zeit zu bewahren.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Diese Foundation basiert auf einem Wirkstoff, der auf zentrale zelluläre Mechanismen wirkt, die mit gesundem Altern in Verbindung stehen.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Hyaluronsäure · 200 mg · Erhöht viskoelastische Eigenschaften der Gelenkflüssigkeit. Unterstützt gleitende Gelenkmechanik.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>immunity-formula</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützt eine stabile und ausgewogene Immunfunktion im Alltag
+Eine stabile Immunfunktion entsteht aus dem Zusammenspiel von Abwehr, Regulation und Schutz vor oxidativem Stress. Vitamin C unterstützt antioxidative Schutzmechanismen, während Vitamin D3, Zink, Selen und Kupfer an der Feinabstimmung der Immunantwort beteiligt sind. So bleibt das Immunsystem im Alltag reaktionsfähig, ohne aus dem Gleichgewicht zu geraten.
+Hilft, chronische Entzündungsbelastung zu regulieren und immunologische Balance zu fördern
+Mit zunehmendem Alter kann eine niedriggradige, chronische Entzündungsaktivität entstehen, die als Inflammaging bezeichnet wird und das Immunsystem dauerhaft beansprucht. Liposomales Quercetin unterstützt zelluläre Prozesse, die an der Regulation entzündlicher Signale beteiligt sind, während Vitamin D3 und Selen zur immunologischen Balance beitragen.
+Fördert die natürliche Abwehrfähigkeit ohne unspezifische Überstimulation
+Eine funktionierende Abwehr braucht Training, nicht Überreizung. Beta-Glucane unterstützen die natürliche Reaktionsfähigkeit des Immunsystems, ohne es unspezifisch zu aktivieren. Ergänzt durch ausgewählte Mikronährstoffe entsteht eine Abwehr, die angepasst und kontrolliert reagieren kann.
+Unterstützt langfristige Immunresilienz und gesundes Altern
+Mit zunehmendem Alter verändern sich immunologische Anforderungen. Antioxidative Mikronährstoffe, ausgewogene Immunmodulation und die Unterstützung zellulärer Schutzmechanismen tragen dazu bei, die Widerstandsfähigkeit des Immunsystems langfristig zu erhalten. So entsteht eine stabile Grundlage für gesundes Altern.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Immunity⁺ die Immunantwort moduliert und zelluläre Abwehrmechanismen kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen werden die enthaltenen Mikronährstoffe in bestehende Prozesse der Immunabwehr integriert. Vitamin C, Zink, Selen und Beta-Glucane unterstützen grundlegende Funktionen der angeborenen Immunantwort. Spürbare Veränderungen sind in dieser frühen Phase nicht zwingend zu erwarten, viele Menschen nehmen jedoch ein stabileres körperliches Grundgefühl wahr.
+4 Wochen
+Mit fortgesetzter Einnahme etabliert sich die unterstützende Wirkung auf zentrale Immun- und Regulationsprozesse. Vitamin D3, Quercetin und Beta-Glucane begleiten die Feinabstimmung der Immunantwort, während Spurenelemente zur normalen Funktion von Immunzellen beitragen. Im Alltag zeigt sich dies häufig in einer besseren Belastbarkeit gegenüber saisonalen oder alltäglichen Herausforderungen.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Versorgung greifen Abwehr- und Regulationsmechanismen verlässlicher ineinander. Die Immunantwort wirkt weniger reaktiv und besser abgestimmt. Viele Anwender berichten in dieser Phase von einer insgesamt stabileren Widerstandskraft, insbesondere in Zeiten erhöhter Belastung oder wechselnder Umweltfaktoren.
+6 Monate
+IMMUNE⁺ entfaltet seine Stärke vor allem als langfristige Unterstützung der Immunregulation. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als ein insgesamt robusteres Gleichgewicht zwischen Abwehr und Regulation. Die kontinuierliche Versorgung mit zentralen Mikronährstoffen trägt dazu bei, die Immunfunktion über die Zeit stabil zu begleiten.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Immunity⁺ wurde entwickelt, um zentrale Immunfunktionen zu unterstützen und die langfristige Immunbalance zu fördern.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Quercetin · 120 mg · Moduliert inflammaging-assoziierte Signalwege. Reguliert entzündliche Zellantworten im Alter.
+Beta-Glucan · 100 mg · Aktiviert Mustererkennungsrezeptoren des Immunsystems. Unterstützt trainierte Immunantworten.
+Zink · 15 mg · Reguliert zelluläre Signalwege der Immunantwort. Unterstützt Funktion immunologischer Enzymsysteme.
+Kupfer · 0,5 mg · Bestandteil antioxidativer Metalloenzyme. Beteiligt an zellulären Immunfunktionen.
+Vitamin D3 (Cholecalciferol) · 50 µg · Moduliert angeborene und adaptive Immunantwort. Unterstützt immunologische Balanceprozesse.
+Vitamin K2 (MK-7) · 100 µg · Moduliert inflammationsassoziierte Signalprozesse. Beeinflusst altersabhängige Gefäß- und Zellprozesse.
+Selen · 55 µg · Ermöglicht selenabhängige antioxidative Enzymaktivität. Beeinflusst immunologische Redoxbalance.
+Vitamin C (Ascorbinsäure) · 250 mg · Ermöglicht enzymatische Kollagensynthese. Kofaktor kollagenabhängiger Gewebestruktur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>kreatin-pulver</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützt Muskelkraft und körperliche Leistungsfähigkeit im Alltag
+Muskelkraft ist eine zentrale Voraussetzung für Leistungsfähigkeit im täglichen Leben. Kreatin unterstützt die schnelle Energiebereitstellung in der Muskulatur und trägt so dazu bei, körperliche Belastungen effizienter zu bewältigen. Das unterstützt Kraft und Stabilität bei alltäglichen Bewegungen.
+Hilft, Energie bei Belastung schnell verfügbar zu machen
+Bei kurzfristiger, intensiver Belastung steigt der Energiebedarf der Muskulatur stark an. Kreatin unterstützt die Regeneration von ATP, der unmittelbaren Energiequelle der Muskelzellen. So kann Energie bei körperlicher Beanspruchung schneller bereitgestellt werden.
+Fördert den Erhalt von Muskelmasse und funktioneller Beweglichkeit
+Muskelmasse ist entscheidend für Kraft, Stabilität und Beweglichkeit. Kreatin unterstützt muskuläre Funktion und Anpassungsprozesse, insbesondere bei zunehmendem Alter. Dadurch kann der Erhalt funktioneller Muskelstruktur gefördert werden.
+Unterstützt langfristige körperliche Selbstständigkeit und gesundes Altern
+Körperliche Selbstständigkeit beruht auf Muskelkraft, Stabilität und Beweglichkeit über die Zeit. Die gezielte Unterstützung muskulärer Energiesysteme trägt dazu bei, diese Fähigkeiten langfristig zu erhalten. So entsteht eine verlässliche Grundlage für gesundes Altern.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Kreatin die intrazelluläre Energieverfügbarkeit und körperliche Leistungsfähigkeit kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+Bereits in den ersten Tagen beginnt Kreatin, sich in Muskel- und Nervenzellen anzureichern. Die schnelle Energiebereitstellung über ATP kann effizienter ablaufen. Viele Menschen nehmen in dieser Phase bei körperlicher Belastung ein etwas kräftigeres, stabileres Leistungsgefühl wahr, insbesondere bei kurzen, intensiven Bewegungen oder Trainingseinheiten.
+4 Wochen
+Mit fortgesetzter Einnahme sind die Kreatinspeicher in der Muskulatur zunehmend gesättigt. Kraft, Schnellenergie und Belastbarkeit können sich spürbarer verbessern. Im Alltag zeigt sich dies häufig in mehr Stabilität bei körperlichen Aufgaben, besserer Leistungsfähigkeit beim Training und weniger schneller Ermüdung.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Anwendung greifen energetische und muskuläre Anpassungsprozesse verlässlicher ineinander. Kreatin unterstützt den Erhalt von Muskelmasse und funktioneller Kraft, was sich positiv auf Beweglichkeit und körperliche Belastbarkeit auswirken kann. Viele Anwender berichten in dieser Phase von mehr Sicherheit und Leistungsreserve bei alltäglichen Bewegungen.
+6 Monate
+Kreatin entfaltet seine Wirkung besonders über die langfristige Unterstützung muskulärer Energiesysteme. Nach mehreren Monaten steht weniger der einzelne Leistungszuwachs im Vordergrund als der Erhalt von Kraft, Funktion und körperlicher Selbstständigkeit. Die kontinuierliche Unterstützung der muskulären Energieversorgung trägt dazu bei, altersbedingtem Kraftverlust strukturell zu begegnen.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Diese Foundation basiert auf einem Wirkstoff, der auf zentrale zelluläre Mechanismen wirkt, die mit gesundem Altern in Verbindung stehen.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Kreatinmonohydrat · 5.000 mg · Unterstützt schnelle Energieverfügbarkeit bei Belastung. Unterstützt Erhalt funktioneller Muskelmasse. Verbessert muskuläre Leistungsfähigkeit bei Intensität.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>men-formula</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützt entzündungsbezogene Balance und zelluläre Stabilität im Alter
+Mit zunehmendem Alter nehmen beim männlichen Körper niedriggradige Entzündungsaktivität und oxidative Belastung besonders in stoffwechselaktiven Geweben zu. Liposomales Curcumin wirkt auf entzündungsassoziierte Signalwege, während Granatapfel-Polyphenole und Lycopin oxidativen Stress abpuffern und die strukturelle Stabilität von Zellen unterstützen. Damit werden zentrale Treiber altersbedingter Zellschädigung adressiert, die beim Mann früh funktionell relevant werden.
+Fördert die mitochondriale Energieversorgung und körperliche Vitalität
+Der altersbedingte Rückgang der mitochondrialen Funktion zählt beim Mann zu den früh dominanten Mechanismen biologischen Alterns. Ubiquinol, die bioaktive Form von Coenzym Q10, übernimmt eine Schlüsselrolle in der mitochondrialen Atmungskette und unterstützt die effiziente ATP-Synthese. Magnesium ergänzt diese Prozesse und stabilisiert die zelluläre Energieverfügbarkeit in Geweben mit hohem Energiebedarf, wie Muskulatur und Herz.
+Trägt zur hormonellen und regulatorischen Stabilität bei
+Beim männlichen Altern verändert sich weniger der Hormonspiegel als die Präzision hormoneller Signalübertragung. Zink ist an der Funktion zahlreicher hormonabhängiger Enzyme und Rezeptoren beteiligt, während Vitamin D3 als hormonähnlicher Signalstoff regulatorische Prozesse unterstützt. Magnesium trägt zur Stabilität neuroendokriner Regelkreise bei und begleitet die altersbedingte Veränderung hormoneller Signalachsen, ohne aktiv einzugreifen.
+Unterstützt langfristige Leistungsfähigkeit und gesundes Altern
+Gesundes Altern beim Mann erfordert die gleichzeitige Stabilisierung zentraler biologischer Systeme: kontrollierte Entzündungsaktivität, funktionierende mitochondriale Energiegewinnung und präzise hormonelle Signalübertragung. Die kombinierte Unterstützung dieser Prozesse trägt dazu bei, körperliche Leistungsfähigkeit und strukturelle Stabilität über die Zeit zu erhalten und altersbedingtem Funktionsverlust gezielt entgegenzuwirken.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Men⁺ hormonelle Balance, Zellschutz und geschlechtsspezifische Stoffwechselfunktionen kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen werden die enthaltenen Mikronährstoffe und Pflanzenstoffe in bestehende Regulationsprozesse eingebunden. Curcumin, Granatapfel-Polyphenole und Lycopin wirken auf entzündungs- und oxidationsbezogene Signalwege, während Ubiquinol unmittelbar in die mitochondriale Energiegewinnung integriert wird. Spürbare Veränderungen sind in dieser frühen Phase nicht zwingend zu erwarten, manche Männer nehmen jedoch ein stabileres Energiegefühl oder weniger körperliche Ermüdung wahr.
+4 Wochen
+Mit fortgesetzter Einnahme beginnen sich die unterstützten Prozesse deutlicher zu stabilisieren. Die mitochondriale Energieversorgung kann gleichmäßiger ablaufen, während entzündungsbezogene Belastungen besser reguliert werden. Im Alltag zeigt sich dies häufig in konstanterer Leistungsfähigkeit, besserer Belastbarkeit und einem ausgeglicheneren körperlichen Grundgefühl.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Anwendung greifen Energie-, Entzündungs- und Regulationsmechanismen verlässlicher ineinander. Viele Anwender berichten in dieser Phase von stabilerer körperlicher Leistungsfähigkeit, verbesserter Erholung und einer insgesamt robusteren Belastbarkeit im Alltag. Hormonelle Signalprozesse wirken häufig präziser abgestimmt, ohne stimulierend einzugreifen.
+6 Monate
+MEN⁺ entfaltet seine Wirkung vor allem langfristig über die Unterstützung zentraler biologischer Systeme, die beim männlichen Altern früh relevant werden. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als ein insgesamt stabiles Leistungsniveau. Die kontinuierliche Begleitung von Energieversorgung, entzündungsbezogener Balance und hormoneller Regulation trägt dazu bei, körperliche Vitalität und funktionelle Stabilität über die Zeit zu erhalten.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Men⁺ wurde entwickelt, um zentrale physiologische Prozesse beim Mann zu unterstützen und die körperliche Leistungsfähigkeit sowie hormonelle Balance im Alltag zu fördern.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Ubiquinol (aktiviertes Q10) · 100 mg · Unterstützt die mitochondriale Energieproduktion Trägt zum Schutz vor oxidativem Stress bei Umgeht Umwandlung zu bioaktiver Q10-Form
+Magnesium · 45 mg · Beteiligt an neuromuskulärer Signalübertragung. Moduliert neuronale Erregbarkeit.
+Zink · 10 mg · Reguliert zelluläre Signalwege der Immunantwort. Unterstützt Funktion immunologischer Enzymsysteme.
+Lycopin · 15 mg · Neutralisiert reaktive Sauerstoffspezies. Schützt lipidhaltige Zellstrukturen.
+Curcumin (liposomal) · 150 mg · Moduliert NF-κB-abhängige Signalwege. Beeinflusst entzündungsassoziierte Enzymaktivität.
+Punicalagine (Granatapfel-Extrakt) · 250 mg · Puffert oxidativen Zellstress ab. Unterstützt strukturelle Zellintegrität.
+Vitamin D3 (Cholecalciferol) · 50 µg · Moduliert angeborene und adaptive Immunantwort. Unterstützt immunologische Balanceprozesse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>metabolism-formula</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützt einen aktiven Stoffwechsel und eine effiziente Energieverwertung
+Berberin unterstützt zentrale Stoffwechselwege, die für eine effiziente Nutzung von Energie entscheidend sind. In Kombination mit Glycin trägt es dazu bei, metabolische Prozesse im Gleichgewicht zu halten. So kann Energie strukturierter und gezielter verwertet werden.
+Fördert die körpereigene Energieproduktion auf Zellebene
+Ubiquinol ist eine bioaktive Form von Coenzym Q10 und spielt eine Schlüsselrolle in der zellulären Energiegewinnung. Es unterstützt die Funktion der Mitochondrien, in denen Energie entsteht. Dadurch kann die körpereigene Energieproduktion zuverlässig aufrechterhalten werden.
+Hilft dem Körper, flexibel auf Belastung und Energiebedarf zu reagieren
+Glycin unterstützt regulatorische Prozesse, die an Stressverarbeitung und metabolischer Anpassung beteiligt sind. Berberin ergänzt diese Wirkung, indem es die metabolische Flexibilität fördert. So kann der Körper besser auf wechselnde Anforderungen reagieren.
+Unterstützt nachhaltige Leistungsfähigkeit und gesundes Altern
+Ein stabiler Stoffwechsel ist entscheidend für Leistungsfähigkeit über die Zeit. Die gezielte Kombination ausgewählter Inhaltsstoffe unterstützt zentrale Prozesse, die Energie, Regeneration und Belastbarkeit im Gleichgewicht halten. So entsteht eine nachhaltige Grundlage für gesundes Altern.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Metabolism⁺ deinen Energiestoffwechsel und zelluläre Funktionen kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen beginnt der Körper, die enthaltenen Wirkstoffe in bestehende Stoffwechselprozesse zu integrieren. Berberin wirkt auf regulatorische Abläufe im Glukose- und Energiestoffwechsel, während Ubiquinol unmittelbar in mitochondriale Prozesse eingebunden wird. Spürbare Veränderungen sind in dieser frühen Phase nicht zwingend zu erwarten, manche Menschen nehmen jedoch ein ruhigeres Energiegefühl oder eine stabilere Verdauung wahr.
+4 Wochen
+Mit fortgesetzter Einnahme beginnen sich die regulierenden Effekte auf den Stoffwechsel deutlicher zu etablieren. Energie wird häufig gleichmäßiger über den Tag verfügbar, ohne stimulierende Spitzen. Im Alltag kann sich dies in weniger ausgeprägten Leistungstiefs, besserer Belastbarkeit nach Mahlzeiten oder einem insgesamt ausgeglicheneren Energieverlauf zeigen.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Anwendung greifen die unterstützten Stoffwechsel- und Energieprozesse verlässlicher ineinander. Berberin trägt zur stabileren metabolischen Regulation bei, Ubiquinol unterstützt die zelluläre Energiegewinnung, während Glycin regenerative und ausgleichende Prozesse begleitet. Viele Anwender berichten in dieser Phase von einem konsistenteren Leistungsniveau und einer verbesserten Anpassungsfähigkeit an Alltag und Stress.
+6 Monate
+Die Wirkung entfaltet sich vor allem langfristig als integrierter Ansatz zur Unterstützung von Stoffwechsel, Energieverwertung und zellulärer Belastbarkeit. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als ein insgesamt stabileres inneres Gleichgewicht. Die kontinuierliche Begleitung zentraler Regulationsprozesse trägt dazu bei, Stoffwechselgesundheit und Leistungsfähigkeit über die Zeit zu erhalten.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Metabolism⁺ wurde entwickelt, um zentrale Stoffwechselprozesse zu unterstützen und die zelluläre Energiegewinnung effizienter zu machen.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>L-Glycin · 1000 mg · Beteiligt an zellulären Reparaturprozessen. Liefert Glycin für Glutathion-Aufbau.
+Berberinextrakt · 500 mg · Fördert metabolische Balance
+Ubiquinol · 200 mg · Unterstützt die mitochondriale Energieproduktion Trägt zum Schutz vor oxidativem Stress bei
+Piperin · 5 mg · Verbessert die Bioverfügbarkeit anderer Wirkstoffe</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>mobility-formula</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützt Beweglichkeit und Gelenkkomfort im Alltag
+Hyaluronsäure unterstützt die Gleitfähigkeit der Gelenkstrukturen und damit die Beweglichkeit im Alltag. MSM ergänzt diese Wirkung durch seine Rolle im Bindegewebsstoffwechsel. So kann sich Bewegung spürbar leichter und angenehmer anfühlen.
+Hilft, strukturelle Belastbarkeit von Gelenken und Bindegewebe zu erhalten
+Vitamin C trägt zur normalen Kollagenbildung für Knorpel, Knochen und Bindegewebe bei. MSM unterstützt strukturelle Prozesse im Gewebe. Dadurch entsteht Stabilität dort, wo Gelenke im Alltag belastet werden.
+Begleitet die natürliche Regulation entzündlicher Prozesse bei körperlicher Belastung
+Curcumin und Boswellia serrata unterstützen Prozesse, die an der physiologischen Entzündungsregulation beteiligt sind. Sie helfen dem Körper, Belastungsreaktionen einzuordnen und auszugleichen. So können Gelenkstrukturen auch unter Beanspruchung im Gleichgewicht bleiben.
+Unterstützt langfristige Mobilität und gesundes Altern
+Beweglichkeit über die Zeit beruht auf struktureller Stabilität und einer ausgewogenen Belastungsregulation. Die gezielte Kombination ausgewählter Inhaltsstoffe unterstützt diese Systeme in ihrem Zusammenspiel. So entsteht eine verlässliche Grundlage für langfristige Mobilität und gesundes Altern.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Mobility⁺ Gelenkfunktion, Beweglichkeit und entzündungsmodulierende Prozesse kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützung, wenn Bewegung gefordert ist
+Mobility⁺ wurde entwickelt, um Gelenke, Bindegewebe und Beweglichkeit gezielt zu unterstützen, insbesondere in Phasen erhöhter körperlicher Belastung oder eingeschränkter Bewegungsfreiheit. Viele Anwender integrieren AGILE⁺ bewusst über mehrere Wochen oder Monate in ihren Alltag, etwa während intensiver Trainingsphasen, bei gesteigerter Beanspruchung oder zur strukturellen Unterstützung. Je nach individuellem Empfinden und Belastung kann die Einnahme flexibel angepasst werden. Pausen oder eine phasenweise Anwendung sind dabei ebenso Teil eines bewussten Umgangs wie eine längere Nutzung bei anhaltendem Bedarf. Entscheidend ist nicht die Dauer, sondern die gezielte Unterstützung in den Momenten, in denen der Körper sie braucht.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Mobility⁺ wurde entwickelt, um zentrale Funktionen von Gelenken und Bindegewebe zu unterstützen und die Beweglichkeit im Alltag zu fördern.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Hyaluronsäure · 50 mg · Erhöht viskoelastische Eigenschaften der Gelenkflüssigkeit. Unterstützt gleitende Gelenkmechanik.
+MSM (Methylsulfonylmethan) · 300 mg · Liefert bioverfügbaren organischen Schwefel. Beteiligt an Bindegewebs-Stoffwechselprozessen.
+Vitamin C (Ascorbinsäure) · 250 mg · Ermöglicht enzymatische Kollagensynthese. Kofaktor kollagenabhängiger Gewebestruktur.
+Curcumin (liposomal) · 250 mg · Moduliert NF-κB-abhängige Signalwege. Beeinflusst entzündungsassoziierte Enzymaktivität.
+Boswellia serrata Extrakt (AKBA-standardisiert) · 200 mg · Hemmt 5-Lipoxygenase-Signalwege. Moduliert leukotrienabhängige Prozesse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>omega-3-kapseln</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützt Herzgesundheit und Gefäßfunktion im Alltag
+Omega-3-Fettsäuren sind Bestandteil der Zellmembranen im Herz-Kreislauf-System. Sie unterstützen physiologische Prozesse, die für eine normale Herzfunktion und die Elastizität der Gefäße relevant sind. So trägt Omega-3 zur kardiovaskulären Stabilität im Alltag bei.
+Fördert Konzentration, mentale Klarheit und Gehirnleistung
+Das Gehirn besteht zu einem hohen Anteil aus Fettsäuren, insbesondere DHA. Omega-3 unterstützt die Struktur neuronaler Zellmembranen und die Signalübertragung zwischen Nervenzellen. So können Konzentrationsfähigkeit und mentale Klarheit gezielt unterstützt werden.
+Unterstützt entzündungsbezogene Balance und langfristige Zellgesundheit
+Omega-3-Fettsäuren sind an der Regulation entzündungsbezogener Signalprozesse auf Zellebene beteiligt. Sie unterstützen die Balance zwischen Belastung und Regeneration. Dadurch wird eine stabile Grundlage für langfristige Zellgesundheit geschaffen.
+Liefert hochdosiertes Omega-3 in hochwertiger rTG-Form für optimale Aufnahme
+Die rTG-Form kommt der natürlichen Struktur von Fettsäuren besonders nahe und unterstützt deren Aufnahme im Körper. In hochdosierter Form steht Omega-3 so effizient für zentrale Zell- und Gewebeprozesse zur Verfügung. Das macht die Qualität der Versorgung spürbar.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Omega-3 die Funktion von Zellmembranen sowie entzündungsregulierende Prozesse kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen werden EPA und DHA in Zellmembranen eingebaut, insbesondere in Geweben mit hohem Umsatz wie Blutgefäßen, Nervenzellen und Immunzellen. Auf struktureller Ebene beginnen Anpassungen der Membraneigenschaften. Spürbare Effekte sind in dieser frühen Phase nicht zwingend zu erwarten, manche Menschen nehmen jedoch ein ruhigeres körperliches oder mentales Grundgefühl wahr.
+4 Wochen
+Mit fortgesetzter Einnahme etabliert sich die Versorgung mit Omega-3-Fettsäuren deutlicher in den Zellmembranen. Prozesse der Gefäßfunktion, neuronalen Signalübertragung und entzündungsbezogenen Regulation können gleichmäßiger ablaufen. Im Alltag zeigt sich dies häufig in stabilerer Konzentration, mentaler Klarheit oder einem insgesamt ausgeglicheneren Leistungsgefühl.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Versorgung greifen die membranbasierten Effekte verlässlicher ineinander. Die Balance entzündungsbezogener Prozesse kann sich stabilisieren, während Herz-Kreislauf- und Gehirnfunktionen strukturell besser unterstützt werden. Viele Anwender berichten in dieser Phase von konstanterer mentaler Leistungsfähigkeit und einem robusteren körperlichen Grundgefühl.
+6 Monate
+Omega-3 entfaltet seine Wirkung vor allem langfristig über die kontinuierliche Integration in Zellmembranen. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als eine insgesamt verbesserte funktionelle Stabilität von Herz, Gehirn und Zellen. Die dauerhafte Versorgung mit EPA und DHA trägt dazu bei, Zellgesundheit, Gefäßfunktion und mentale Leistungsfähigkeit über die Zeit zu erhalten.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Diese Foundation basiert auf einem Wirkstoff, der auf zentrale zelluläre Mechanismen wirkt, die mit gesundem Altern in Verbindung stehen.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Eicosapentaensäure (EPA) · 1.500 mg · Beeinflusst zelluläre Regenerationssignale.
+Docosahexaensäure (DHA) · 750 mg · Unterstützt synaptische Signalübertragung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>recovery-formula</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützt Regeneration und Belastbarkeit nach körperlicher Beanspruchung
+Körperliche Belastung führt zu mikroskopischen Gewebereizen und erhöhtem Stress auf Zellebene. Curcumin, Boswellia und Ingwer wirken auf Prozesse, die an der Einordnung und Verarbeitung dieser Belastungen beteiligt sind. So kann Regeneration geordnet ablaufen und der Körper nach Beanspruchung schneller in ein funktionelles Gleichgewicht zurückfinden.
+Schützt Zellen vor oxidativem Stress bei erhöhter Beanspruchung
+Intensive Bewegung, Training und Alltagsstress erhöhen die oxidative Belastung der Zellen. Vitamin E, Astaxanthin und Pterostilben unterstützen antioxidative Schutzmechanismen, die freie Radikale abpuffern und Zellstrukturen stabilisieren. Dadurch bleibt die zelluläre Integrität auch unter wiederholter Belastung besser erhalten.
+Fördert entzündungsbezogene Balance im Bewegungsapparat
+Entzündungsreaktionen sind ein natürlicher Bestandteil von Anpassung und Regeneration, müssen jedoch kontrolliert bleiben. Curcumin und Boswellia unterstützen Signalwege, die an der physiologischen Regulation entzündungsbezogener Prozesse beteiligt sind. So wird eine Balance zwischen Belastung und Erholung begünstigt, ohne natürliche Anpassungsmechanismen zu blockieren.
+Unterstützt nachhaltige Vitalität und gesundes Altern
+Nachhaltige Leistungsfähigkeit entsteht nicht durch kurzfristige Erholung, sondern durch die Fähigkeit des Körpers, Belastungen wiederholt zu verarbeiten. Die abgestimmte Kombination ausgewählter Inhaltsstoffe begleitet Regeneration, Zellschutz und Regulationsprozesse im Zusammenspiel. So entsteht eine verlässliche Grundlage für funktionelle Resilienz und körperliche Belastbarkeit über die Zeit.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Recovery⁺ Regenerationsprozesse nach Belastung unterstützt und zelluläre Erholung kurz- und langfristig fördern kann.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützung, wenn Regeneration gefragt ist
+Recovery⁺ wurde entwickelt, um Regenerationsprozesse und Belastungsverarbeitung gezielt zu begleiten, insbesondere in Phasen erhöhter körperlicher Beanspruchung oder wiederholter Belastung. Viele Anwender integrieren RECOV⁺ bewusst über mehrere Wochen in ihren Alltag, etwa während intensiver Trainingsphasen, bei hoher körperlicher oder beruflicher Belastung oder wenn Erholung strukturierter unterstützt werden soll. Je nach individuellem Empfinden und Beanspruchung kann die Einnahme flexibel angepasst werden. Pausen oder eine phasenweise Anwendung sind dabei ebenso Teil eines bewussten Umgangs wie eine längere Nutzung bei anhaltendem Bedarf. Entscheidend ist nicht die Dauer, sondern die gezielte Unterstützung in den Phasen, in denen Regeneration und Ausgleich besonders gefordert sind.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Recovery⁺ wurde entwickelt, um zentrale Regenerationsprozesse zu unterstützen und die zelluläre Erholung nach körperlicher und metabolischer Belastung zu fördern.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Curcumin (liposomal) · 200 mg · Moduliert NF-κB-abhängige Signalwege. Beeinflusst entzündungsassoziierte Enzymaktivität.
+Vitamin E (D-alpha-Tocopherol) · 20 mg · Unterbricht lipidperoxidative Kettenreaktionen. Schützt membranständige Zellstrukturen.
+Boswellia serrata Extrakt (AKBA-standardisiert) · 200 mg · Hemmt 5-Lipoxygenase-Signalwege. Moduliert leukotrienabhängige Prozesse.
+Ingwerextrakt · 150 mg · Beeinflusst COX- und LOX-assoziierte Signalprozesse. Moduliert zelluläre Stress- und Adaptationssignale.
+Pterostilben · 100 mg · Aktiviert antioxidative Schutzsignalwege. Beeinflusst zelluläre Stressresilienz.
+Astaxanthin · 4 mg · Schützt Zellmembranen vor oxidativem Stress. Stabilisiert mitochondriale Redoxbalance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>sleep-formula</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Erleichtert das Einschlafen und unterstützt einen ruhigen Übergang in die Nacht
+L-Theanin unterstützt Prozesse, die mentale Aktivität am Abend beruhigen und den Übergang in den Schlaf erleichtern. Magnesium-Bisglycinat ergänzt diese Wirkung, indem es zur Entspannung des Nervensystems beiträgt. So entsteht ein natürlicher Übergang in die Nacht.
+Fördert tiefen, stabilen Schlaf für bessere nächtliche Regeneration
+Magnesium spielt eine zentrale Rolle bei der Regulation von Nerven- und Muskelaktivität während des Schlafs. In gut verfügbarer Form unterstützt es die Stabilität nächtlicher Ruhephasen. Das schafft die Voraussetzung für kontinuierliche Regeneration.
+Hilft, mentale Unruhe und körperliche Anspannung am Abend zu reduzieren
+L-Theanin und Apigenin unterstützen ausgleichende Prozesse im Nervensystem. Sie tragen dazu bei, körperliche Anspannung zu lösen und das innere Gleichgewicht am Abend zu stabilisieren. Dadurch kann Entspannung tiefer und nachhaltiger wirken.
+Unterstützt erholtes Aufwachen und nachhaltige Leistungsfähigkeit am Tag
+Erholsamer Schlaf ist entscheidend für Leistungsfähigkeit über die Zeit. Die gezielte Kombination ausgewählter Inhaltsstoffe unterstützt zentrale Prozesse, die nächtliche Regeneration und innere Balance fördern. So entsteht eine verlässliche Grundlage für nachhaltige Leistungsfähigkeit im Alltag.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Sleep⁺ das neurochemische Gleichgewicht am Abend unterstützt und die Qualität erholsamen Schlafs kurz- und langfristig fördern kann.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+Bereits in den ersten Tagen unterstützen Magnesium-Bisglycinat, L-Theanin und Apigenin aus Kamille ausgleichende Prozesse im Nervensystem. Viele Menschen nehmen schnelleres Abschalten am Abend, weniger innere Unruhe oder ein ruhigeres Einschlafen wahr. Die Wirkung setzt meist ohne sedierende Effekte ein.
+4 Wochen
+Mit fortgesetzter Einnahme über mehrere Wochen kann sich der Schlaf-Wach-Rhythmus weiter stabilisieren. Einschlafen fällt häufig konstanter, nächtliche Unruhe kann abnehmen. Im Alltag zeigt sich dies oft in erholterem Aufwachen und besserer mentaler Belastbarkeit am Tag.
+3 Monate
+Bei Bedarf über einen längeren Zeitraum eingesetzt, kann SLEEP⁺ dazu beitragen, stressbedingte Schlafmuster nachhaltig zu regulieren. Viele Anwender berichten, dass sie in dieser Phase weniger auf äußere Hilfen angewiesen sind und Schlaf wieder als verlässliche Ressource wahrnehmen.
+6 Monate
+Nach mehreren Monaten regelmäßiger Nutzung entscheiden sich viele Menschen bewusst für eine Pause oder eine situative Anwendung. Die zuvor unterstützten Entspannungs- und Regulationsprozesse können dabei als Grundlage für stabileren Schlaf erhalten bleiben.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Sleep⁺ wurde entwickelt, um zentrale Prozesse der Schlafregulation zu unterstützen und die nächtliche Erholung des Nervensystems zu fördern.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>L-Theanin · 200 mg · Unterstützt neurophysiologische Balance. Trägt zur Unterstützung der Schlafqualität bei.
+Magnesium-Bisglycinat · 600 mg · Unterstützt die normale Nervenfunktion. Trägt zur Stabilität nächtlicher Ruhephasen bei
+Apigenin · 50 mg · Unterstützt ausgleichende Prozesse im Nervensystem Trägt zur Entspannungsregulation bei</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>spermidin-kapseln</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Stärkt die natürliche Zellreinigung und -erneuerung
+Zellen müssen beschädigte oder nicht mehr benötigte Bestandteile regelmäßig abbauen, um funktionsfähig zu bleiben. Spermidin unterstützt die physiologischen Prozesse, die diese zelluläre Reinigung und Erneuerung ermöglichen. So bleibt die Zellfunktion langfristig erhalten.
+Fördert funktionelle Zellqualität statt kurzfristiger Effekte
+Gesunde Zellen zeichnen sich durch strukturelle Integrität und Erneuerungsfähigkeit aus, nicht durch kurzfristige Aktivierung. Spermidin wirkt auf Prozesse, die die Qualität und Funktionalität von Zellen über die Zeit beeinflussen. Der Fokus liegt auf nachhaltiger Zellfunktion statt schneller Effekte.
+Hochdosiertes Spermidin (6 mg) zur Aktivierung zellulärer Autophagie-Prozesse
+Autophagie ist ein zentraler Prozess der zellulären Selbstreinigung. Spermidin ist an der Regulation dieser Mechanismen beteiligt und unterstützt autophagiebezogene Signalwege. In hochdosierter Form steht es gezielt für diese Prozesse zur Verfügung.
+Unterstützt nachhaltige Vitalität und gesundes Altern
+Langfristige Vitalität beruht auf der Fähigkeit von Zellen, sich selbst zu erneuern und funktionsfähig zu bleiben. Die Unterstützung autophagieabhängiger Prozesse trägt dazu bei, zelluläre Stabilität über die Zeit zu bewahren. So entsteht eine verlässliche Grundlage für gesundes Altern.</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Spermidin zelluläre Reinigungsprozesse aktiviert und Mechanismen gesunder Langlebigkeit kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen wird Spermidin in zelluläre Signalwege eingebunden, die mit Autophagie und zellulärer Selbstreinigung verbunden sind. Auf Zellebene werden Prozesse angestoßen, die beschädigte oder nicht mehr benötigte Zellbestandteile erfassen. Spürbare Effekte sind in dieser frühen Phase nicht zu erwarten, da die Wirkung nicht akut, sondern strukturell ansetzt.
+4 Wochen
+Mit fortgesetzter Einnahme können sich autophagiebezogene Prozesse im Zellstoffwechsel stabilisieren. Zellen beginnen, Erneuerungs- und Recyclingmechanismen verlässlicher zu nutzen. Im Alltag äußert sich dies nicht als einzelner Effekt, sondern eher als ein ruhiges, stabiles Funktionsniveau ohne kurzfristige Peaks.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Versorgung greifen Prozesse der Zellreinigung und -erneuerung deutlich geordneter ineinander. Die funktionelle Qualität von Zellen kann sich verbessern, da belastende oder dysfunktionale Strukturen konsequenter abgebaut werden. Viele Anwender beschreiben diese Phase als ein insgesamt robusteres inneres Gleichgewicht.
+6 Monate
+Spermidin entfaltet seine Wirkung vor allem langfristig über die Unterstützung autophagieabhängiger Erhaltungsprozesse. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als die strukturelle Erneuerungsfähigkeit von Zellen. Die kontinuierliche Begleitung dieser Prozesse trägt dazu bei, Zellfunktion und Stabilität über die Zeit zu bewahren und gesundes Altern zu unterstützen.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Diese Foundation basiert auf einem Wirkstoff, der auf zentrale zelluläre Mechanismen wirkt, die mit gesundem Altern in Verbindung stehen.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Spermidin (aus Weizenkeimextrakt) · 6 mg · Aktiviert autophagieabhängige Zellreinigung. Unterstützt zelluläre Qualitätskontrolle. Erhält strukturelle Zellintegrität über die Zeit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>sulphoraphan-kapseln</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Hilft, oxidativen und entzündlichen Belastungen im Alltag besser zu begegnen
+Oxidative und entzündliche Belastungen entstehen täglich durch Stoffwechsel, Umwelt und Lebensstil. Sulphoraphane unterstützt regulatorische Prozesse, die an der Einordnung und Kontrolle dieser Belastungen beteiligt sind. So kann das zelluläre Gleichgewicht auch unter alltäglicher Beanspruchung besser gewahrt bleiben.
+Stärkt zelluläre Anpassungsfähigkeit bei Umwelt- und Alltagsstress
+Zellen müssen sich kontinuierlich an wechselnde Anforderungen anpassen. Sulphoraphane unterstützt Signalwege, die an Stress- und Anpassungsreaktionen beteiligt sind. Dadurch können Zellen flexibler auf Umwelt- und Alltagsstress reagieren.
+Fördert die körpereigenen Schutzmechanismen der Zellen
+Zellen verfügen über eigene Schutzsysteme, um ihre Funktion langfristig zu erhalten. Sulphoraphane unterstützt Signalwege, die an der Regulation zellulärer Schutzmechanismen beteiligt sind, darunter auch der Nrf2-abhängige Stressantwortweg. So können körpereigene Schutzsysteme gezielt unterstützt werden.
+Unterstützt langfristige Zellgesundheit und gesundes Altern
+Langfristige Gesundheit beginnt auf Zellebene. Die Unterstützung von Schutz- und Anpassungsmechanismen trägt dazu bei, Funktion und Stabilität über die Zeit zu bewahren. So entsteht eine verlässliche Grundlage für gesundes Altern.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Sulphoraphan zelluläre Schutzmechanismen aktiviert und körpereigene Entgiftungsprozesse kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen wird Sulforaphan in zelluläre Signalwege eingebunden, die mit Schutz- und Anpassungsprozessen zusammenhängen. Auf Zellebene werden Mechanismen aktiviert, die den Umgang mit oxidativen und entzündlichen Belastungen unterstützen. Spürbare Effekte sind in dieser frühen Phase nicht zwingend zu erwarten, viele Menschen nehmen jedoch ein stabileres körperliches Grundgefühl wahr.
+4 Wochen
+Mit fortgesetzter Einnahme beginnen sich die unterstützten Schutz- und Regulationsprozesse deutlicher zu etablieren. Zellen reagieren häufig gelassener auf alltägliche Belastungen durch Umwelt, Stress oder Stoffwechselaktivität. Im Alltag zeigt sich dies weniger als einzelner Effekt, sondern als insgesamt ausgeglichenere Belastbarkeit.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Versorgung greifen Anpassungs- und Schutzmechanismen verlässlicher ineinander. Die Fähigkeit der Zellen, auf wechselnde Anforderungen zu reagieren und innere Balance zu wahren, kann sich spürbar stabilisieren. Viele Anwender berichten in dieser Phase von einem robusteren Gefühl im Umgang mit Stress und Belastung.
+6 Monate
+Sulforaphan entfaltet seine Wirkung vor allem langfristig über die Unterstützung körpereigener Schutz- und Anpassungssysteme. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als eine insgesamt verbesserte zelluläre Widerstandskraft. Die kontinuierliche Begleitung dieser Prozesse trägt dazu bei, Zellfunktion und Stabilität über die Zeit zu erhalten.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Diese Foundation basiert auf einem Wirkstoff, der auf zentrale zelluläre Mechanismen wirkt, die mit gesundem Altern in Verbindung stehen.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Sulforaphan · 6mg · Induziert antioxidative Schutzenzyme. Beeinflusst inflammationsassoziierte Signaltransduktion. Unterstützt zelluläre Stressanpassung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>taurin-kapseln</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Hilft dem Körper, besser mit Stress und Belastung umzugehen
+Taurin ist in hohen Konzentrationen im Nervensystem vorhanden und an der Regulation neuronaler Erregbarkeit beteiligt. Es unterstützt Prozesse, die Reizüberflutung und Stressreaktionen ausgleichen. So kann der Körper Belastungen kontrollierter verarbeiten.
+Fördert eine ausgeglichene Energie- und Stoffwechselregulation
+Taurin beeinflusst den Calciumhaushalt der Zellen und unterstützt damit zentrale Stoffwechsel- und Energieprozesse. Diese Regulation ist entscheidend für eine effiziente Zusammenarbeit von Nerven, Muskeln und Mitochondrien. Dadurch kann Energie bedarfsgerechter bereitgestellt werden.
+Stärkt zelluläre Stabilität und innere Balance
+Taurin spielt eine zentrale Rolle bei der Osmoregulation und Stabilisierung von Zellmembranen. Es hilft Zellen, ihr inneres Gleichgewicht auch unter wechselnden Bedingungen aufrechtzuerhalten. So wird strukturelle und funktionelle Zellstabilität unterstützt.
+Unterstützt langfristige Resilienz und gesundes Altern
+Zelluläre Resilienz beruht auf stabilen Membranen, regulierter Reizverarbeitung und funktionierendem Energiestoffwechsel. Die Unterstützung dieser grundlegenden Systeme trägt dazu bei, Belastbarkeit und Anpassungsfähigkeit über die Zeit zu bewahren. So entsteht eine verlässliche Grundlage für gesundes Altern.</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Taurin die neuronale Signalübertragung und die zelluläre Stressregulation kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen wird Taurin in zelluläre Prozesse eingebunden, die für Reizverarbeitung, Osmoregulation und Stressantwort relevant sind. Besonders im Nervensystem unterstützt Taurin ausgleichende Mechanismen. Viele Menschen nehmen in dieser Phase ein ruhigeres inneres Grundgefühl oder eine bessere Stressverträglichkeit wahr, ohne sedierende Effekte.
+4 Wochen
+Mit fortgesetzter Einnahme können sich die stabilisierenden Effekte auf Energie- und Stoffwechselregulation deutlicher zeigen. Die Zusammenarbeit von Nerven, Muskulatur und Energiesystemen wirkt häufig besser abgestimmt. Im Alltag äußert sich dies oft in gleichmäßigerer Leistungsfähigkeit und weniger abrupten Erschöpfungsphasen.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Versorgung greifen die unterstützten Regulations- und Stabilitätsprozesse verlässlicher ineinander. Zellmembranen, Reizverarbeitung und Energieverwertung sind besser aufeinander abgestimmt. Viele Anwender berichten in dieser Phase von erhöhter Belastbarkeit, besserer Erholung und einem insgesamt stabileren Leistungsniveau.
+6 Monate
+Taurin entfaltet seine Wirkung vor allem langfristig über die Unterstützung grundlegender zellulärer Stabilitätsmechanismen. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als eine insgesamt verbesserte Resilienz. Die kontinuierliche Begleitung dieser Prozesse trägt dazu bei, körperliche und mentale Leistungsfähigkeit über die Zeit zu erhalten.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Diese Foundation basiert auf einem Wirkstoff, der auf zentrale zelluläre Mechanismen wirkt, die mit gesundem Altern in Verbindung stehen.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>L-Taurin · 1.500 mg · Reguliert neuronale Calcium-Homöostase Moduliert inhibitorische Neurotransmission</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>trimethylglycin-kapseln</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Unterstützt zentrale Methylierungs- und Regulationsprozesse im Stoffwechsel
+Methylierungsprozesse steuern grundlegende Stoffwechsel- und Regulationsfunktionen im Körper. Sie sind entscheidend für Zellfunktion, Energieverwertung und innere Balance. Die gezielte Unterstützung dieser Prozesse trägt zu einer stabilen metabolischen Steuerung bei.
+Trägt zu einem ausgeglichenen Homocystein-Stoffwechsel bei
+Ein regulierter Homocystein-Stoffwechsel ist ein wichtiger Marker für metabolische und kardiovaskuläre Balance. Bestimmte Mikronährstoffe unterstützen die Umwandlung und den Abbau von Homocystein im Rahmen physiologischer Prozesse. So kann ein ausgeglichenes inneres Milieu erhalten bleiben.
+Fördert metabolische Stabilität und zelluläre Balance
+Wenn zentrale Regulationsprozesse zuverlässig ineinandergreifen, bleibt der Stoffwechsel auch auf Zellebene stabil. Die Unterstützung dieser Abstimmung hilft, Belastungen auszugleichen und funktionelle Balance zu bewahren. So kann metabolische Stabilität langfristig erhalten bleiben.
+Unterstützt langfristige Vitalität und gesundes Altern
+Langfristige Vitalität basiert auf funktionierenden Regulationssystemen und einem stabilen Stoffwechsel. Die Kombination ausgewählter Inhaltsstoffe unterstützt diese Prozesse in ihrem Zusammenspiel. So entsteht eine verlässliche Grundlage für gesundes Altern und nachhaltige Leistungsfähigkeit.</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie TMG den Methylstoffwechsel und die zelluläre Stoffwechselbalance kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen steht Trimethylglycin dem Körper als Methylgruppenlieferant für zentrale Stoffwechselprozesse zur Verfügung. Auf zellulärer Ebene werden Methylierungsreaktionen unterstützt, die an Energieverwertung und Zellschutz beteiligt sind. Spürbare Effekte sind in dieser frühen Phase nicht zwingend zu erwarten, manche Menschen nehmen jedoch ein stabileres inneres Grundgefühl oder eine ruhigere metabolische Reaktion auf Belastung wahr.
+4 Wochen
+In den ersten Tagen steht Trimethylglycin dem Körper als Methylgruppenlieferant für zentrale Stoffwechselprozesse zur Verfügung. Auf zellulärer Ebene werden Methylierungsreaktionen unterstützt, die an Energieverwertung und Zellschutz beteiligt sind. Spürbare Effekte sind in dieser frühen Phase nicht zwingend zu erwarten, manche Menschen nehmen jedoch ein stabileres inneres Grundgefühl oder eine ruhigere metabolische Reaktion auf Belastung wahr.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Versorgung greifen metabolische Steuerungsmechanismen verlässlicher ineinander. Ein ausgeglichener Homocystein-Stoffwechsel kann dazu beitragen, zelluläre Balance und funktionelle Stabilität zu erhalten. Viele Anwender berichten in dieser Phase von besserer Belastbarkeit und einem insgesamt robusteren Stoffwechselgefühl.
+6 Monate
+TMG entfaltet seine Wirkung vor allem langfristig über die Unterstützung zentraler Regulationssysteme im Stoffwechsel. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als eine insgesamt stabilere metabolische Basis. Die kontinuierliche Begleitung von Methylierungsprozessen trägt dazu bei, Vitalität und Leistungsfähigkeit über die Zeit zu erhalten.</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Diese Foundation basiert auf einem Wirkstoff, der auf zentrale zelluläre Mechanismen wirkt, die mit gesundem Altern in Verbindung stehen.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Trimethylglycin · 1.000 mg · Liefert Methylgruppen für Methylierungsreaktionen. Fördert Remethylierung von Homocystein. Unterstützt metabolische Regulationsprozesse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>ubiquinol-q10-kapseln</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Fördert Leistungsfähigkeit bei nachlassender körpereigener Q10-Produktion
+Mit zunehmendem Alter nimmt die körpereigene Q10-Produktion ab, während der Bedarf an zellulärer Energie steigt. In dieser Phase kann herkömmliches Q10 an Wirksamkeit verlieren. Direkt verfügbares Ubiquinol trägt dazu bei, die Energieversorgung gezielt dort zu stärken, wo sie zunehmend gefordert ist.
+Liefert direkt verfügbares Ubiquinol statt herkömmlichem Q10
+Ubiquinol ist die bioaktive Form von Coenzym Q10, die dem Körper unmittelbar zur Verfügung steht. Im Gegensatz zu herkömmlichem Q10 entfällt der Umwandlungsschritt in die aktive Form. So steht der Wirkstoff direkt für zentrale Energieprozesse bereit.
+Trägt zu einer effizienten mitochondrialen Energiegewinnung bei
+Ubiquinol ist ein zentraler Bestandteil der mitochondrialen Atmungskette, in der zelluläre Energie entsteht. Es ist an Prozessen beteiligt, die für eine zuverlässige ATP-Produktion erforderlich sind. Dadurch kann die Energiegewinnung auf Zellebene effizient und stabil ablaufen.
+Unterstützt nachhaltige Vitalität und gesundes Altern
+Zelluläre Energie ist eine wesentliche Voraussetzung für langfristige Leistungsfähigkeit. Die gezielte Unterstützung mitochondrialer Prozesse hilft, körperliche und mentale Energie über die Zeit zu bewahren. So entsteht eine stabile Basis für gesundes Altern.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Entdecke, wie Ubiquinol (aktiviertes Q10) die mitochondriale Energieversorgung und den antioxidativen Zellschutz kurz- und langfristig unterstützen kann.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>1 Woche
+In den ersten Tagen steht Ubiquinol dem Körper unmittelbar als bioaktive Form von Coenzym Q10 zur Verfügung. Auf zellulärer Ebene wird es in bestehende mitochondriale Prozesse eingebunden. Spürbare Effekte sind in dieser Phase nicht zwingend zu erwarten, manche Menschen berichten jedoch von einem etwas stabileren Energiegefühl ohne stimulierende Wirkung.
+4 Wochen
+Mit fortgesetzter Einnahme integriert sich Ubiquinol zunehmend in die mitochondriale Energiegewinnung. Energie wird häufig gleichmäßiger bereitgestellt, insbesondere bei alltäglicher körperlicher oder mentaler Belastung. Viele Anwender nehmen in dieser Phase wahr, dass sie sich weniger schnell erschöpft fühlen und Belastungen konstanter bewältigen können.
+3 Monate
+Nach mehreren Wochen kontinuierlicher Versorgung wirkt sich die verbesserte mitochondriale Funktion deutlicher aus. Körperliche Leistungsfähigkeit, Ausdauer im Alltag und subjektive Belastbarkeit können sich spürbar stabilisieren. Energie steht nicht nur kurzfristig zur Verfügung, sondern bleibt über den Tag hinweg verlässlicher abrufbar.
+6 Monate
+Ubiquinol entfaltet seine Wirkung vor allem langfristig über die Unterstützung zentraler Energieprozesse in den Zellen. Nach mehreren Monaten steht weniger ein einzelner Effekt im Vordergrund als ein insgesamt robusteres Energieniveau. Die kontinuierliche Versorgung trägt dazu bei, altersbedingten Veränderungen der körpereigenen Q10-Produktion strukturell zu begegnen und Vitalität über die Zeit zu erhalten.</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Diese Foundation basiert auf einem Wirkstoff, der auf zentrale zelluläre Mechanismen wirkt, die mit gesundem Altern in Verbindung stehen.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Ubiquinol (aktiviertes Q10) · 100 mg · Unterstützt die mitochondriale Energieproduktion Trägt zum Schutz vor oxidativem Stress bei Umgeht Umwandlung zu bioaktiver Q10-Form</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>